<commit_message>
More correct map between types.
</commit_message>
<xml_diff>
--- a/example/example.xlsx
+++ b/example/example.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\GitHub\calendar-Excel\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6283E66-BBBA-49D3-86D4-01E051E73881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A973754D-266E-4501-81A7-1B2EA39AB0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D027B85-A559-4D5D-8EB5-E53AEF402827}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -425,13 +425,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E5178B5-5BF6-4934-8AF1-976F0CFC01B0}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" cm="1">
         <f t="array" ref="B2">[1]!CalendarSetAsOfDate()</f>
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Factor out enum for error codes.
</commit_message>
<xml_diff>
--- a/example/example.xlsx
+++ b/example/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\GitHub\calendar-Excel\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A973754D-266E-4501-81A7-1B2EA39AB0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{959AA6CE-DE9A-48FA-BEC3-DA9C02F4ADAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D027B85-A559-4D5D-8EB5-E53AEF402827}"/>
   </bookViews>
@@ -432,7 +432,7 @@
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" cm="1">
         <f t="array" ref="B2">[1]!CalendarSetAsOfDate()</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Parse the date on the C++ side.
</commit_message>
<xml_diff>
--- a/example/example.xlsx
+++ b/example/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\GitHub\calendar-Excel\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{959AA6CE-DE9A-48FA-BEC3-DA9C02F4ADAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1049CFF-7D3E-4BC6-BBD8-FB7204EE4DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D027B85-A559-4D5D-8EB5-E53AEF402827}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="191029" calcMode="manual" calcOnSave="0"/>
+  <calcPr calcId="191029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -60,8 +60,24 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -89,8 +105,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,12 +444,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E5178B5-5BF6-4934-8AF1-976F0CFC01B0}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B2"/>
+  <dimension ref="B2:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B2" cm="1">
-        <f t="array" ref="B2">[1]!CalendarSetAsOfDate()</f>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="1">
+        <f ca="1">TODAY()</f>
+        <v>46117</v>
+      </c>
+      <c r="C2" s="2" cm="1">
+        <f t="array" aca="1" ref="C2" ca="1">[1]!CalendarSetAsOfDate(B2)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a DLL function for IsBusinessDay.
</commit_message>
<xml_diff>
--- a/example/example.xlsx
+++ b/example/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\GitHub\calendar-Excel\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1049CFF-7D3E-4BC6-BBD8-FB7204EE4DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1E64CB-DE3C-4047-BB76-91A98A00A143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D027B85-A559-4D5D-8EB5-E53AEF402827}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="191029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
+  <calcPr calcId="191029" calcMode="manual" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -56,6 +56,26 @@
     </bk>
   </cellMetadata>
 </metadata>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>AsOfDate</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>IsBusinessDay</t>
+  </si>
+  <si>
+    <t>Calendar</t>
+  </si>
+  <si>
+    <t>America/ANBIMA</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -105,10 +125,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -137,6 +158,7 @@
       <sheetName val="Sheet1"/>
     </sheetNames>
     <definedNames>
+      <definedName name="CalendarIsBusinessDay"/>
       <definedName name="CalendarSetAsOfDate"/>
     </definedNames>
     <sheetDataSet>
@@ -444,20 +466,166 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E5178B5-5BF6-4934-8AF1-976F0CFC01B0}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B2:C2"/>
+  <dimension ref="B2:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="1">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="1">
         <f ca="1">TODAY()</f>
         <v>46117</v>
       </c>
-      <c r="C2" s="2" cm="1">
-        <f t="array" aca="1" ref="C2" ca="1">[1]!CalendarSetAsOfDate(B2)</f>
+      <c r="C3" s="2" cm="1">
+        <f t="array" aca="1" ref="C3" ca="1">[1]!CalendarSetAsOfDate(B3)</f>
         <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>46113</v>
+      </c>
+      <c r="F3" t="b" cm="1">
+        <f t="array" ref="F3">[1]!CalendarIsBusinessDay(E3,$B$6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E4" s="1">
+        <f>E3+1</f>
+        <v>46114</v>
+      </c>
+      <c r="F4" t="b" cm="1">
+        <f t="array" ref="F4">[1]!CalendarIsBusinessDay(E4,$B$6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" ref="E5:E15" si="0">E4+1</f>
+        <v>46115</v>
+      </c>
+      <c r="F5" t="b" cm="1">
+        <f t="array" ref="F5">[1]!CalendarIsBusinessDay(E5,$B$6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>46116</v>
+      </c>
+      <c r="F6" t="b" cm="1">
+        <f t="array" ref="F6">[1]!CalendarIsBusinessDay(E6,$B$6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>46117</v>
+      </c>
+      <c r="F7" t="b" cm="1">
+        <f t="array" ref="F7">[1]!CalendarIsBusinessDay(E7,$B$6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>46118</v>
+      </c>
+      <c r="F8" t="b" cm="1">
+        <f t="array" ref="F8">[1]!CalendarIsBusinessDay(E8,$B$6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>46119</v>
+      </c>
+      <c r="F9" t="b" cm="1">
+        <f t="array" ref="F9">[1]!CalendarIsBusinessDay(E9,$B$6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>46120</v>
+      </c>
+      <c r="F10" t="b" cm="1">
+        <f t="array" ref="F10">[1]!CalendarIsBusinessDay(E10,$B$6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>46121</v>
+      </c>
+      <c r="F11" t="b" cm="1">
+        <f t="array" ref="F11">[1]!CalendarIsBusinessDay(E11,$B$6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>46122</v>
+      </c>
+      <c r="F12" t="b" cm="1">
+        <f t="array" ref="F12">[1]!CalendarIsBusinessDay(E12,$B$6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E13" s="1">
+        <f t="shared" si="0"/>
+        <v>46123</v>
+      </c>
+      <c r="F13" t="b" cm="1">
+        <f t="array" ref="F13">[1]!CalendarIsBusinessDay(E13,$B$6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E14" s="1">
+        <f t="shared" si="0"/>
+        <v>46124</v>
+      </c>
+      <c r="F14" t="b" cm="1">
+        <f t="array" ref="F14">[1]!CalendarIsBusinessDay(E14,$B$6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E15" s="1">
+        <f t="shared" si="0"/>
+        <v>46125</v>
+      </c>
+      <c r="F15" t="b" cm="1">
+        <f t="array" ref="F15">[1]!CalendarIsBusinessDay(E15,$B$6)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add a DLL function for CountBusinessDays.
</commit_message>
<xml_diff>
--- a/example/example.xlsx
+++ b/example/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\GitHub\calendar-Excel\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1E64CB-DE3C-4047-BB76-91A98A00A143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D605D959-3F3C-4DDB-AA9E-D28E9D50B09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D027B85-A559-4D5D-8EB5-E53AEF402827}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="191029" calcMode="manual" calcOnSave="0"/>
+  <calcPr calcId="191029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>AsOfDate</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t>America/ANBIMA</t>
+  </si>
+  <si>
+    <t>CountBusinessDays</t>
   </si>
 </sst>
 </file>
@@ -158,6 +161,7 @@
       <sheetName val="Sheet1"/>
     </sheetNames>
     <definedNames>
+      <definedName name="CalendarCountBusinessDays"/>
       <definedName name="CalendarIsBusinessDay"/>
       <definedName name="CalendarSetAsOfDate"/>
     </definedNames>
@@ -466,15 +470,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E5178B5-5BF6-4934-8AF1-976F0CFC01B0}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B2:F15"/>
+  <dimension ref="B2:H15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -484,8 +489,11 @@
       <c r="F2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1">
         <f ca="1">TODAY()</f>
         <v>46117</v>
@@ -497,22 +505,26 @@
       <c r="E3" s="1">
         <v>46113</v>
       </c>
-      <c r="F3" t="b" cm="1">
+      <c r="F3" s="2" t="b" cm="1">
         <f t="array" ref="F3">[1]!CalendarIsBusinessDay(E3,$B$6)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H3" s="2" cm="1">
+        <f t="array" aca="1" ref="H3" ca="1">[1]!CalendarCountBusinessDays(E3,E15,B6)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E4" s="1">
         <f>E3+1</f>
         <v>46114</v>
       </c>
-      <c r="F4" t="b" cm="1">
+      <c r="F4" s="2" t="b" cm="1">
         <f t="array" ref="F4">[1]!CalendarIsBusinessDay(E4,$B$6)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -520,12 +532,12 @@
         <f t="shared" ref="E5:E15" si="0">E4+1</f>
         <v>46115</v>
       </c>
-      <c r="F5" t="b" cm="1">
+      <c r="F5" s="2" t="b" cm="1">
         <f t="array" ref="F5">[1]!CalendarIsBusinessDay(E5,$B$6)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
@@ -533,97 +545,97 @@
         <f t="shared" si="0"/>
         <v>46116</v>
       </c>
-      <c r="F6" t="b" cm="1">
+      <c r="F6" s="2" t="b" cm="1">
         <f t="array" ref="F6">[1]!CalendarIsBusinessDay(E6,$B$6)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E7" s="1">
         <f t="shared" si="0"/>
         <v>46117</v>
       </c>
-      <c r="F7" t="b" cm="1">
+      <c r="F7" s="2" t="b" cm="1">
         <f t="array" ref="F7">[1]!CalendarIsBusinessDay(E7,$B$6)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E8" s="1">
         <f t="shared" si="0"/>
         <v>46118</v>
       </c>
-      <c r="F8" t="b" cm="1">
+      <c r="F8" s="2" t="b" cm="1">
         <f t="array" ref="F8">[1]!CalendarIsBusinessDay(E8,$B$6)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E9" s="1">
         <f t="shared" si="0"/>
         <v>46119</v>
       </c>
-      <c r="F9" t="b" cm="1">
+      <c r="F9" s="2" t="b" cm="1">
         <f t="array" ref="F9">[1]!CalendarIsBusinessDay(E9,$B$6)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E10" s="1">
         <f t="shared" si="0"/>
         <v>46120</v>
       </c>
-      <c r="F10" t="b" cm="1">
+      <c r="F10" s="2" t="b" cm="1">
         <f t="array" ref="F10">[1]!CalendarIsBusinessDay(E10,$B$6)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E11" s="1">
         <f t="shared" si="0"/>
         <v>46121</v>
       </c>
-      <c r="F11" t="b" cm="1">
+      <c r="F11" s="2" t="b" cm="1">
         <f t="array" ref="F11">[1]!CalendarIsBusinessDay(E11,$B$6)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E12" s="1">
         <f t="shared" si="0"/>
         <v>46122</v>
       </c>
-      <c r="F12" t="b" cm="1">
+      <c r="F12" s="2" t="b" cm="1">
         <f t="array" ref="F12">[1]!CalendarIsBusinessDay(E12,$B$6)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E13" s="1">
         <f t="shared" si="0"/>
         <v>46123</v>
       </c>
-      <c r="F13" t="b" cm="1">
+      <c r="F13" s="2" t="b" cm="1">
         <f t="array" ref="F13">[1]!CalendarIsBusinessDay(E13,$B$6)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E14" s="1">
         <f t="shared" si="0"/>
         <v>46124</v>
       </c>
-      <c r="F14" t="b" cm="1">
+      <c r="F14" s="2" t="b" cm="1">
         <f t="array" ref="F14">[1]!CalendarIsBusinessDay(E14,$B$6)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E15" s="1">
         <f t="shared" si="0"/>
         <v>46125</v>
       </c>
-      <c r="F15" t="b" cm="1">
+      <c r="F15" s="2" t="b" cm="1">
         <f t="array" ref="F15">[1]!CalendarIsBusinessDay(E15,$B$6)</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Make example more informative.
</commit_message>
<xml_diff>
--- a/example/example.xlsx
+++ b/example/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\GitHub\calendar-Excel\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47B4CE2-8849-4ACE-A952-EB90AB9959B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DA0E6A-295A-410B-B1B9-62AB2464FA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D027B85-A559-4D5D-8EB5-E53AEF402827}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>AsOfDate</t>
   </si>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t>Calendar</t>
-  </si>
-  <si>
-    <t>America/ANBIMA</t>
   </si>
   <si>
     <t>CountBusinessDays</t>
@@ -111,12 +108,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -131,11 +134,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,7 +492,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" t="s">
         <v>1</v>
@@ -497,7 +501,7 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
@@ -513,11 +517,11 @@
         <v>45597</v>
       </c>
       <c r="F3" s="2" t="b" cm="1">
-        <f t="array" ref="F3">[1]!CalendarIsBusinessDay(E3,$B$6)</f>
+        <f t="array" aca="1" ref="F3" ca="1">[1]!CalendarIsBusinessDay(E3,$B$6)</f>
         <v>1</v>
       </c>
       <c r="H3" s="2" cm="1">
-        <f t="array" ref="H3">[1]!CalendarCountBusinessDays(E3,E32,B6)</f>
+        <f t="array" aca="1" ref="H3" ca="1">[1]!CalendarCountBusinessDays(E3,E32,B6)</f>
         <v>19</v>
       </c>
     </row>
@@ -527,7 +531,7 @@
         <v>45598</v>
       </c>
       <c r="F4" s="2" t="b" cm="1">
-        <f t="array" ref="F4">[1]!CalendarIsBusinessDay(E4,$B$6)</f>
+        <f t="array" aca="1" ref="F4" ca="1">[1]!CalendarIsBusinessDay(E4,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -536,24 +540,25 @@
         <v>3</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" ref="E5:E33" si="0">E4+1</f>
+        <f t="shared" ref="E5:E32" si="0">E4+1</f>
         <v>45599</v>
       </c>
       <c r="F5" s="2" t="b" cm="1">
-        <f t="array" ref="F5">[1]!CalendarIsBusinessDay(E5,$B$6)</f>
+        <f t="array" aca="1" ref="F5" ca="1">[1]!CalendarIsBusinessDay(E5,$B$6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>4</v>
+      <c r="B6" s="3" t="str">
+        <f ca="1">IF(C3=0,"America/ANBIMA","")</f>
+        <v>America/ANBIMA</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="0"/>
         <v>45600</v>
       </c>
       <c r="F6" s="2" t="b" cm="1">
-        <f t="array" ref="F6">[1]!CalendarIsBusinessDay(E6,$B$6)</f>
+        <f t="array" aca="1" ref="F6" ca="1">[1]!CalendarIsBusinessDay(E6,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -563,7 +568,7 @@
         <v>45601</v>
       </c>
       <c r="F7" s="2" t="b" cm="1">
-        <f t="array" ref="F7">[1]!CalendarIsBusinessDay(E7,$B$6)</f>
+        <f t="array" aca="1" ref="F7" ca="1">[1]!CalendarIsBusinessDay(E7,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -573,7 +578,7 @@
         <v>45602</v>
       </c>
       <c r="F8" s="2" t="b" cm="1">
-        <f t="array" ref="F8">[1]!CalendarIsBusinessDay(E8,$B$6)</f>
+        <f t="array" aca="1" ref="F8" ca="1">[1]!CalendarIsBusinessDay(E8,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -583,7 +588,7 @@
         <v>45603</v>
       </c>
       <c r="F9" s="2" t="b" cm="1">
-        <f t="array" ref="F9">[1]!CalendarIsBusinessDay(E9,$B$6)</f>
+        <f t="array" aca="1" ref="F9" ca="1">[1]!CalendarIsBusinessDay(E9,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -593,7 +598,7 @@
         <v>45604</v>
       </c>
       <c r="F10" s="2" t="b" cm="1">
-        <f t="array" ref="F10">[1]!CalendarIsBusinessDay(E10,$B$6)</f>
+        <f t="array" aca="1" ref="F10" ca="1">[1]!CalendarIsBusinessDay(E10,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -603,7 +608,7 @@
         <v>45605</v>
       </c>
       <c r="F11" s="2" t="b" cm="1">
-        <f t="array" ref="F11">[1]!CalendarIsBusinessDay(E11,$B$6)</f>
+        <f t="array" aca="1" ref="F11" ca="1">[1]!CalendarIsBusinessDay(E11,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -613,7 +618,7 @@
         <v>45606</v>
       </c>
       <c r="F12" s="2" t="b" cm="1">
-        <f t="array" ref="F12">[1]!CalendarIsBusinessDay(E12,$B$6)</f>
+        <f t="array" aca="1" ref="F12" ca="1">[1]!CalendarIsBusinessDay(E12,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -623,7 +628,7 @@
         <v>45607</v>
       </c>
       <c r="F13" s="2" t="b" cm="1">
-        <f t="array" ref="F13">[1]!CalendarIsBusinessDay(E13,$B$6)</f>
+        <f t="array" aca="1" ref="F13" ca="1">[1]!CalendarIsBusinessDay(E13,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -633,7 +638,7 @@
         <v>45608</v>
       </c>
       <c r="F14" s="2" t="b" cm="1">
-        <f t="array" ref="F14">[1]!CalendarIsBusinessDay(E14,$B$6)</f>
+        <f t="array" aca="1" ref="F14" ca="1">[1]!CalendarIsBusinessDay(E14,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -643,7 +648,7 @@
         <v>45609</v>
       </c>
       <c r="F15" s="2" t="b" cm="1">
-        <f t="array" ref="F15">[1]!CalendarIsBusinessDay(E15,$B$6)</f>
+        <f t="array" aca="1" ref="F15" ca="1">[1]!CalendarIsBusinessDay(E15,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -653,7 +658,7 @@
         <v>45610</v>
       </c>
       <c r="F16" s="2" t="b" cm="1">
-        <f t="array" ref="F16">[1]!CalendarIsBusinessDay(E16,$B$6)</f>
+        <f t="array" aca="1" ref="F16" ca="1">[1]!CalendarIsBusinessDay(E16,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -663,7 +668,7 @@
         <v>45611</v>
       </c>
       <c r="F17" s="2" t="b" cm="1">
-        <f t="array" ref="F17">[1]!CalendarIsBusinessDay(E17,$B$6)</f>
+        <f t="array" aca="1" ref="F17" ca="1">[1]!CalendarIsBusinessDay(E17,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -673,7 +678,7 @@
         <v>45612</v>
       </c>
       <c r="F18" s="2" t="b" cm="1">
-        <f t="array" ref="F18">[1]!CalendarIsBusinessDay(E18,$B$6)</f>
+        <f t="array" aca="1" ref="F18" ca="1">[1]!CalendarIsBusinessDay(E18,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -683,7 +688,7 @@
         <v>45613</v>
       </c>
       <c r="F19" s="2" t="b" cm="1">
-        <f t="array" ref="F19">[1]!CalendarIsBusinessDay(E19,$B$6)</f>
+        <f t="array" aca="1" ref="F19" ca="1">[1]!CalendarIsBusinessDay(E19,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -693,7 +698,7 @@
         <v>45614</v>
       </c>
       <c r="F20" s="2" t="b" cm="1">
-        <f t="array" ref="F20">[1]!CalendarIsBusinessDay(E20,$B$6)</f>
+        <f t="array" aca="1" ref="F20" ca="1">[1]!CalendarIsBusinessDay(E20,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -703,7 +708,7 @@
         <v>45615</v>
       </c>
       <c r="F21" s="2" t="b" cm="1">
-        <f t="array" ref="F21">[1]!CalendarIsBusinessDay(E21,$B$6)</f>
+        <f t="array" aca="1" ref="F21" ca="1">[1]!CalendarIsBusinessDay(E21,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -712,8 +717,8 @@
         <f t="shared" si="0"/>
         <v>45616</v>
       </c>
-      <c r="F22" s="2" t="b" cm="1">
-        <f t="array" ref="F22">[1]!CalendarIsBusinessDay(E22,$B$6)</f>
+      <c r="F22" s="4" t="b" cm="1">
+        <f t="array" aca="1" ref="F22" ca="1">[1]!CalendarIsBusinessDay(E22,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -723,7 +728,7 @@
         <v>45617</v>
       </c>
       <c r="F23" s="2" t="b" cm="1">
-        <f t="array" ref="F23">[1]!CalendarIsBusinessDay(E23,$B$6)</f>
+        <f t="array" aca="1" ref="F23" ca="1">[1]!CalendarIsBusinessDay(E23,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -733,7 +738,7 @@
         <v>45618</v>
       </c>
       <c r="F24" s="2" t="b" cm="1">
-        <f t="array" ref="F24">[1]!CalendarIsBusinessDay(E24,$B$6)</f>
+        <f t="array" aca="1" ref="F24" ca="1">[1]!CalendarIsBusinessDay(E24,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -743,7 +748,7 @@
         <v>45619</v>
       </c>
       <c r="F25" s="2" t="b" cm="1">
-        <f t="array" ref="F25">[1]!CalendarIsBusinessDay(E25,$B$6)</f>
+        <f t="array" aca="1" ref="F25" ca="1">[1]!CalendarIsBusinessDay(E25,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -753,7 +758,7 @@
         <v>45620</v>
       </c>
       <c r="F26" s="2" t="b" cm="1">
-        <f t="array" ref="F26">[1]!CalendarIsBusinessDay(E26,$B$6)</f>
+        <f t="array" aca="1" ref="F26" ca="1">[1]!CalendarIsBusinessDay(E26,$B$6)</f>
         <v>0</v>
       </c>
     </row>
@@ -763,7 +768,7 @@
         <v>45621</v>
       </c>
       <c r="F27" s="2" t="b" cm="1">
-        <f t="array" ref="F27">[1]!CalendarIsBusinessDay(E27,$B$6)</f>
+        <f t="array" aca="1" ref="F27" ca="1">[1]!CalendarIsBusinessDay(E27,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -773,7 +778,7 @@
         <v>45622</v>
       </c>
       <c r="F28" s="2" t="b" cm="1">
-        <f t="array" ref="F28">[1]!CalendarIsBusinessDay(E28,$B$6)</f>
+        <f t="array" aca="1" ref="F28" ca="1">[1]!CalendarIsBusinessDay(E28,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -783,7 +788,7 @@
         <v>45623</v>
       </c>
       <c r="F29" s="2" t="b" cm="1">
-        <f t="array" ref="F29">[1]!CalendarIsBusinessDay(E29,$B$6)</f>
+        <f t="array" aca="1" ref="F29" ca="1">[1]!CalendarIsBusinessDay(E29,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -793,7 +798,7 @@
         <v>45624</v>
       </c>
       <c r="F30" s="2" t="b" cm="1">
-        <f t="array" ref="F30">[1]!CalendarIsBusinessDay(E30,$B$6)</f>
+        <f t="array" aca="1" ref="F30" ca="1">[1]!CalendarIsBusinessDay(E30,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -803,7 +808,7 @@
         <v>45625</v>
       </c>
       <c r="F31" s="2" t="b" cm="1">
-        <f t="array" ref="F31">[1]!CalendarIsBusinessDay(E31,$B$6)</f>
+        <f t="array" aca="1" ref="F31" ca="1">[1]!CalendarIsBusinessDay(E31,$B$6)</f>
         <v>1</v>
       </c>
     </row>
@@ -813,7 +818,7 @@
         <v>45626</v>
       </c>
       <c r="F32" s="2" t="b" cm="1">
-        <f t="array" ref="F32">[1]!CalendarIsBusinessDay(E32,$B$6)</f>
+        <f t="array" aca="1" ref="F32" ca="1">[1]!CalendarIsBusinessDay(E32,$B$6)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete a ToDo item.
</commit_message>
<xml_diff>
--- a/example/example.xlsx
+++ b/example/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\GitHub\calendar-Excel\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DA0E6A-295A-410B-B1B9-62AB2464FA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA59889C-B4A9-41BB-8765-5A194DCE1231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D027B85-A559-4D5D-8EB5-E53AEF402827}"/>
   </bookViews>
@@ -509,9 +509,9 @@
         <f ca="1">TODAY()</f>
         <v>46117</v>
       </c>
-      <c r="C3" s="2" cm="1">
+      <c r="C3" s="2" t="str" cm="1">
         <f t="array" aca="1" ref="C3" ca="1">[1]!CalendarSetAsOfDate(B3)</f>
-        <v>0</v>
+        <v>Set</v>
       </c>
       <c r="E3" s="1">
         <v>45597</v>
@@ -550,7 +550,7 @@
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="str">
-        <f ca="1">IF(C3=0,"America/ANBIMA","")</f>
+        <f ca="1">IF(C3="Set","America/ANBIMA","")</f>
         <v>America/ANBIMA</v>
       </c>
       <c r="E6" s="1">

</xml_diff>